<commit_message>
Omission of 4 participants due to lack of group assignment
ניקוי הקובץ הסופי (באמצעות סקריפט 04 merge) מארבעה נבדקים ללא שיוך קבוצתי ולידי. בנוסף, עדכון קקובץ excluded participants שנמצא בתוך תיקיית lab screening, וציון ארבעת הנבדקים האלו
</commit_message>
<xml_diff>
--- a/Data/lab_screening/participant_excluded_review.xlsx
+++ b/Data/lab_screening/participant_excluded_review.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tulum/Dropbox/Github/Creativity-in-ADHD/Data/lab_screening/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38388D68-35EB-B74A-ABE1-37348033622A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{149235C9-5B3C-4344-BAA9-2CABF03AC9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1620" windowWidth="28800" windowHeight="14480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="45">
   <si>
     <t>subjectid</t>
   </si>
@@ -143,6 +143,21 @@
   </si>
   <si>
     <t>exlusion_reason</t>
+  </si>
+  <si>
+    <t>missing group assignment</t>
+  </si>
+  <si>
+    <t>YyLeol</t>
+  </si>
+  <si>
+    <t>fzgsNA</t>
+  </si>
+  <si>
+    <t>95xyap</t>
+  </si>
+  <si>
+    <t>kPjb3e</t>
   </si>
 </sst>
 </file>
@@ -502,12 +517,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="4" width="17.6640625" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.5" customWidth="1"/>
     <col min="9" max="9" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -880,8 +896,40 @@
         <v>7</v>
       </c>
     </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I26" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>